<commit_message>
Fix issues with the npx command
</commit_message>
<xml_diff>
--- a/demo/demo.xlsx
+++ b/demo/demo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\~\Webcellar\.webcellar\demo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\~\Webcellar\demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75725515-4CE5-44F7-816A-8D67C5F8D5D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E27335-113A-435E-AE67-B52599EC5749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{5844D1C2-6B2C-497A-8A2F-C753586316ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5844D1C2-6B2C-497A-8A2F-C753586316ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16692,7 +16692,7 @@
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="9">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="380" row="9">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="9">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -17060,8 +17060,8 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" cm="1">
-        <f t="array" aca="1" ref="A45" ca="1">_xldudf_A_VOLATILESTATEFULRANDOMWALK()</f>
-        <v>8.7975426878857981</v>
+        <f t="array" ref="A45">_xldudf_A_VOLATILESTATEFULRANDOMWALK()</f>
+        <v>0.70081943955346693</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -17122,7 +17122,7 @@
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="str" cm="1">
         <f t="array" ref="A60">_xldudf_A_TIMESTAMP(TRUE)</f>
-        <v>Mon, 06 Apr 2026 04:53:51 GMT</v>
+        <v>Tue, 07 Apr 2026 02:03:28 GMT</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -36982,6 +36982,544 @@
     <sortCondition ref="H1:H1101"/>
   </sortState>
   <mergeCells count="550">
+    <mergeCell ref="B1094:B1095"/>
+    <mergeCell ref="B1096:B1097"/>
+    <mergeCell ref="B1098:B1099"/>
+    <mergeCell ref="B1100:B1101"/>
+    <mergeCell ref="B1082:B1083"/>
+    <mergeCell ref="B1084:B1085"/>
+    <mergeCell ref="B1086:B1087"/>
+    <mergeCell ref="B1088:B1089"/>
+    <mergeCell ref="B1090:B1091"/>
+    <mergeCell ref="B1092:B1093"/>
+    <mergeCell ref="B1070:B1071"/>
+    <mergeCell ref="B1072:B1073"/>
+    <mergeCell ref="B1074:B1075"/>
+    <mergeCell ref="B1076:B1077"/>
+    <mergeCell ref="B1078:B1079"/>
+    <mergeCell ref="B1080:B1081"/>
+    <mergeCell ref="B1058:B1059"/>
+    <mergeCell ref="B1060:B1061"/>
+    <mergeCell ref="B1062:B1063"/>
+    <mergeCell ref="B1064:B1065"/>
+    <mergeCell ref="B1066:B1067"/>
+    <mergeCell ref="B1068:B1069"/>
+    <mergeCell ref="B1046:B1047"/>
+    <mergeCell ref="B1048:B1049"/>
+    <mergeCell ref="B1050:B1051"/>
+    <mergeCell ref="B1052:B1053"/>
+    <mergeCell ref="B1054:B1055"/>
+    <mergeCell ref="B1056:B1057"/>
+    <mergeCell ref="B1034:B1035"/>
+    <mergeCell ref="B1036:B1037"/>
+    <mergeCell ref="B1038:B1039"/>
+    <mergeCell ref="B1040:B1041"/>
+    <mergeCell ref="B1042:B1043"/>
+    <mergeCell ref="B1044:B1045"/>
+    <mergeCell ref="B1022:B1023"/>
+    <mergeCell ref="B1024:B1025"/>
+    <mergeCell ref="B1026:B1027"/>
+    <mergeCell ref="B1028:B1029"/>
+    <mergeCell ref="B1030:B1031"/>
+    <mergeCell ref="B1032:B1033"/>
+    <mergeCell ref="B1010:B1011"/>
+    <mergeCell ref="B1012:B1013"/>
+    <mergeCell ref="B1014:B1015"/>
+    <mergeCell ref="B1016:B1017"/>
+    <mergeCell ref="B1018:B1019"/>
+    <mergeCell ref="B1020:B1021"/>
+    <mergeCell ref="B998:B999"/>
+    <mergeCell ref="B1000:B1001"/>
+    <mergeCell ref="B1002:B1003"/>
+    <mergeCell ref="B1004:B1005"/>
+    <mergeCell ref="B1006:B1007"/>
+    <mergeCell ref="B1008:B1009"/>
+    <mergeCell ref="B986:B987"/>
+    <mergeCell ref="B988:B989"/>
+    <mergeCell ref="B990:B991"/>
+    <mergeCell ref="B992:B993"/>
+    <mergeCell ref="B994:B995"/>
+    <mergeCell ref="B996:B997"/>
+    <mergeCell ref="B974:B975"/>
+    <mergeCell ref="B976:B977"/>
+    <mergeCell ref="B978:B979"/>
+    <mergeCell ref="B980:B981"/>
+    <mergeCell ref="B982:B983"/>
+    <mergeCell ref="B984:B985"/>
+    <mergeCell ref="B962:B963"/>
+    <mergeCell ref="B964:B965"/>
+    <mergeCell ref="B966:B967"/>
+    <mergeCell ref="B968:B969"/>
+    <mergeCell ref="B970:B971"/>
+    <mergeCell ref="B972:B973"/>
+    <mergeCell ref="B950:B951"/>
+    <mergeCell ref="B952:B953"/>
+    <mergeCell ref="B954:B955"/>
+    <mergeCell ref="B956:B957"/>
+    <mergeCell ref="B958:B959"/>
+    <mergeCell ref="B960:B961"/>
+    <mergeCell ref="B938:B939"/>
+    <mergeCell ref="B940:B941"/>
+    <mergeCell ref="B942:B943"/>
+    <mergeCell ref="B944:B945"/>
+    <mergeCell ref="B946:B947"/>
+    <mergeCell ref="B948:B949"/>
+    <mergeCell ref="B926:B927"/>
+    <mergeCell ref="B928:B929"/>
+    <mergeCell ref="B930:B931"/>
+    <mergeCell ref="B932:B933"/>
+    <mergeCell ref="B934:B935"/>
+    <mergeCell ref="B936:B937"/>
+    <mergeCell ref="B914:B915"/>
+    <mergeCell ref="B916:B917"/>
+    <mergeCell ref="B918:B919"/>
+    <mergeCell ref="B920:B921"/>
+    <mergeCell ref="B922:B923"/>
+    <mergeCell ref="B924:B925"/>
+    <mergeCell ref="B902:B903"/>
+    <mergeCell ref="B904:B905"/>
+    <mergeCell ref="B906:B907"/>
+    <mergeCell ref="B908:B909"/>
+    <mergeCell ref="B910:B911"/>
+    <mergeCell ref="B912:B913"/>
+    <mergeCell ref="B890:B891"/>
+    <mergeCell ref="B892:B893"/>
+    <mergeCell ref="B894:B895"/>
+    <mergeCell ref="B896:B897"/>
+    <mergeCell ref="B898:B899"/>
+    <mergeCell ref="B900:B901"/>
+    <mergeCell ref="B878:B879"/>
+    <mergeCell ref="B880:B881"/>
+    <mergeCell ref="B882:B883"/>
+    <mergeCell ref="B884:B885"/>
+    <mergeCell ref="B886:B887"/>
+    <mergeCell ref="B888:B889"/>
+    <mergeCell ref="B866:B867"/>
+    <mergeCell ref="B868:B869"/>
+    <mergeCell ref="B870:B871"/>
+    <mergeCell ref="B872:B873"/>
+    <mergeCell ref="B874:B875"/>
+    <mergeCell ref="B876:B877"/>
+    <mergeCell ref="B854:B855"/>
+    <mergeCell ref="B856:B857"/>
+    <mergeCell ref="B858:B859"/>
+    <mergeCell ref="B860:B861"/>
+    <mergeCell ref="B862:B863"/>
+    <mergeCell ref="B864:B865"/>
+    <mergeCell ref="B842:B843"/>
+    <mergeCell ref="B844:B845"/>
+    <mergeCell ref="B846:B847"/>
+    <mergeCell ref="B848:B849"/>
+    <mergeCell ref="B850:B851"/>
+    <mergeCell ref="B852:B853"/>
+    <mergeCell ref="B830:B831"/>
+    <mergeCell ref="B832:B833"/>
+    <mergeCell ref="B834:B835"/>
+    <mergeCell ref="B836:B837"/>
+    <mergeCell ref="B838:B839"/>
+    <mergeCell ref="B840:B841"/>
+    <mergeCell ref="B818:B819"/>
+    <mergeCell ref="B820:B821"/>
+    <mergeCell ref="B822:B823"/>
+    <mergeCell ref="B824:B825"/>
+    <mergeCell ref="B826:B827"/>
+    <mergeCell ref="B828:B829"/>
+    <mergeCell ref="B806:B807"/>
+    <mergeCell ref="B808:B809"/>
+    <mergeCell ref="B810:B811"/>
+    <mergeCell ref="B812:B813"/>
+    <mergeCell ref="B814:B815"/>
+    <mergeCell ref="B816:B817"/>
+    <mergeCell ref="B794:B795"/>
+    <mergeCell ref="B796:B797"/>
+    <mergeCell ref="B798:B799"/>
+    <mergeCell ref="B800:B801"/>
+    <mergeCell ref="B802:B803"/>
+    <mergeCell ref="B804:B805"/>
+    <mergeCell ref="B782:B783"/>
+    <mergeCell ref="B784:B785"/>
+    <mergeCell ref="B786:B787"/>
+    <mergeCell ref="B788:B789"/>
+    <mergeCell ref="B790:B791"/>
+    <mergeCell ref="B792:B793"/>
+    <mergeCell ref="B770:B771"/>
+    <mergeCell ref="B772:B773"/>
+    <mergeCell ref="B774:B775"/>
+    <mergeCell ref="B776:B777"/>
+    <mergeCell ref="B778:B779"/>
+    <mergeCell ref="B780:B781"/>
+    <mergeCell ref="B758:B759"/>
+    <mergeCell ref="B760:B761"/>
+    <mergeCell ref="B762:B763"/>
+    <mergeCell ref="B764:B765"/>
+    <mergeCell ref="B766:B767"/>
+    <mergeCell ref="B768:B769"/>
+    <mergeCell ref="B746:B747"/>
+    <mergeCell ref="B748:B749"/>
+    <mergeCell ref="B750:B751"/>
+    <mergeCell ref="B752:B753"/>
+    <mergeCell ref="B754:B755"/>
+    <mergeCell ref="B756:B757"/>
+    <mergeCell ref="B734:B735"/>
+    <mergeCell ref="B736:B737"/>
+    <mergeCell ref="B738:B739"/>
+    <mergeCell ref="B740:B741"/>
+    <mergeCell ref="B742:B743"/>
+    <mergeCell ref="B744:B745"/>
+    <mergeCell ref="B722:B723"/>
+    <mergeCell ref="B724:B725"/>
+    <mergeCell ref="B726:B727"/>
+    <mergeCell ref="B728:B729"/>
+    <mergeCell ref="B730:B731"/>
+    <mergeCell ref="B732:B733"/>
+    <mergeCell ref="B710:B711"/>
+    <mergeCell ref="B712:B713"/>
+    <mergeCell ref="B714:B715"/>
+    <mergeCell ref="B716:B717"/>
+    <mergeCell ref="B718:B719"/>
+    <mergeCell ref="B720:B721"/>
+    <mergeCell ref="B698:B699"/>
+    <mergeCell ref="B700:B701"/>
+    <mergeCell ref="B702:B703"/>
+    <mergeCell ref="B704:B705"/>
+    <mergeCell ref="B706:B707"/>
+    <mergeCell ref="B708:B709"/>
+    <mergeCell ref="B686:B687"/>
+    <mergeCell ref="B688:B689"/>
+    <mergeCell ref="B690:B691"/>
+    <mergeCell ref="B692:B693"/>
+    <mergeCell ref="B694:B695"/>
+    <mergeCell ref="B696:B697"/>
+    <mergeCell ref="B674:B675"/>
+    <mergeCell ref="B676:B677"/>
+    <mergeCell ref="B678:B679"/>
+    <mergeCell ref="B680:B681"/>
+    <mergeCell ref="B682:B683"/>
+    <mergeCell ref="B684:B685"/>
+    <mergeCell ref="B662:B663"/>
+    <mergeCell ref="B664:B665"/>
+    <mergeCell ref="B666:B667"/>
+    <mergeCell ref="B668:B669"/>
+    <mergeCell ref="B670:B671"/>
+    <mergeCell ref="B672:B673"/>
+    <mergeCell ref="B650:B651"/>
+    <mergeCell ref="B652:B653"/>
+    <mergeCell ref="B654:B655"/>
+    <mergeCell ref="B656:B657"/>
+    <mergeCell ref="B658:B659"/>
+    <mergeCell ref="B660:B661"/>
+    <mergeCell ref="B638:B639"/>
+    <mergeCell ref="B640:B641"/>
+    <mergeCell ref="B642:B643"/>
+    <mergeCell ref="B644:B645"/>
+    <mergeCell ref="B646:B647"/>
+    <mergeCell ref="B648:B649"/>
+    <mergeCell ref="B626:B627"/>
+    <mergeCell ref="B628:B629"/>
+    <mergeCell ref="B630:B631"/>
+    <mergeCell ref="B632:B633"/>
+    <mergeCell ref="B634:B635"/>
+    <mergeCell ref="B636:B637"/>
+    <mergeCell ref="B614:B615"/>
+    <mergeCell ref="B616:B617"/>
+    <mergeCell ref="B618:B619"/>
+    <mergeCell ref="B620:B621"/>
+    <mergeCell ref="B622:B623"/>
+    <mergeCell ref="B624:B625"/>
+    <mergeCell ref="B602:B603"/>
+    <mergeCell ref="B604:B605"/>
+    <mergeCell ref="B606:B607"/>
+    <mergeCell ref="B608:B609"/>
+    <mergeCell ref="B610:B611"/>
+    <mergeCell ref="B612:B613"/>
+    <mergeCell ref="B590:B591"/>
+    <mergeCell ref="B592:B593"/>
+    <mergeCell ref="B594:B595"/>
+    <mergeCell ref="B596:B597"/>
+    <mergeCell ref="B598:B599"/>
+    <mergeCell ref="B600:B601"/>
+    <mergeCell ref="B578:B579"/>
+    <mergeCell ref="B580:B581"/>
+    <mergeCell ref="B582:B583"/>
+    <mergeCell ref="B584:B585"/>
+    <mergeCell ref="B586:B587"/>
+    <mergeCell ref="B588:B589"/>
+    <mergeCell ref="B566:B567"/>
+    <mergeCell ref="B568:B569"/>
+    <mergeCell ref="B570:B571"/>
+    <mergeCell ref="B572:B573"/>
+    <mergeCell ref="B574:B575"/>
+    <mergeCell ref="B576:B577"/>
+    <mergeCell ref="B554:B555"/>
+    <mergeCell ref="B556:B557"/>
+    <mergeCell ref="B558:B559"/>
+    <mergeCell ref="B560:B561"/>
+    <mergeCell ref="B562:B563"/>
+    <mergeCell ref="B564:B565"/>
+    <mergeCell ref="B542:B543"/>
+    <mergeCell ref="B544:B545"/>
+    <mergeCell ref="B546:B547"/>
+    <mergeCell ref="B548:B549"/>
+    <mergeCell ref="B550:B551"/>
+    <mergeCell ref="B552:B553"/>
+    <mergeCell ref="B530:B531"/>
+    <mergeCell ref="B532:B533"/>
+    <mergeCell ref="B534:B535"/>
+    <mergeCell ref="B536:B537"/>
+    <mergeCell ref="B538:B539"/>
+    <mergeCell ref="B540:B541"/>
+    <mergeCell ref="B518:B519"/>
+    <mergeCell ref="B520:B521"/>
+    <mergeCell ref="B522:B523"/>
+    <mergeCell ref="B524:B525"/>
+    <mergeCell ref="B526:B527"/>
+    <mergeCell ref="B528:B529"/>
+    <mergeCell ref="B506:B507"/>
+    <mergeCell ref="B508:B509"/>
+    <mergeCell ref="B510:B511"/>
+    <mergeCell ref="B512:B513"/>
+    <mergeCell ref="B514:B515"/>
+    <mergeCell ref="B516:B517"/>
+    <mergeCell ref="B494:B495"/>
+    <mergeCell ref="B496:B497"/>
+    <mergeCell ref="B498:B499"/>
+    <mergeCell ref="B500:B501"/>
+    <mergeCell ref="B502:B503"/>
+    <mergeCell ref="B504:B505"/>
+    <mergeCell ref="B482:B483"/>
+    <mergeCell ref="B484:B485"/>
+    <mergeCell ref="B486:B487"/>
+    <mergeCell ref="B488:B489"/>
+    <mergeCell ref="B490:B491"/>
+    <mergeCell ref="B492:B493"/>
+    <mergeCell ref="B470:B471"/>
+    <mergeCell ref="B472:B473"/>
+    <mergeCell ref="B474:B475"/>
+    <mergeCell ref="B476:B477"/>
+    <mergeCell ref="B478:B479"/>
+    <mergeCell ref="B480:B481"/>
+    <mergeCell ref="B458:B459"/>
+    <mergeCell ref="B460:B461"/>
+    <mergeCell ref="B462:B463"/>
+    <mergeCell ref="B464:B465"/>
+    <mergeCell ref="B466:B467"/>
+    <mergeCell ref="B468:B469"/>
+    <mergeCell ref="B446:B447"/>
+    <mergeCell ref="B448:B449"/>
+    <mergeCell ref="B450:B451"/>
+    <mergeCell ref="B452:B453"/>
+    <mergeCell ref="B454:B455"/>
+    <mergeCell ref="B456:B457"/>
+    <mergeCell ref="B434:B435"/>
+    <mergeCell ref="B436:B437"/>
+    <mergeCell ref="B438:B439"/>
+    <mergeCell ref="B440:B441"/>
+    <mergeCell ref="B442:B443"/>
+    <mergeCell ref="B444:B445"/>
+    <mergeCell ref="B422:B423"/>
+    <mergeCell ref="B424:B425"/>
+    <mergeCell ref="B426:B427"/>
+    <mergeCell ref="B428:B429"/>
+    <mergeCell ref="B430:B431"/>
+    <mergeCell ref="B432:B433"/>
+    <mergeCell ref="B410:B411"/>
+    <mergeCell ref="B412:B413"/>
+    <mergeCell ref="B414:B415"/>
+    <mergeCell ref="B416:B417"/>
+    <mergeCell ref="B418:B419"/>
+    <mergeCell ref="B420:B421"/>
+    <mergeCell ref="B398:B399"/>
+    <mergeCell ref="B400:B401"/>
+    <mergeCell ref="B402:B403"/>
+    <mergeCell ref="B404:B405"/>
+    <mergeCell ref="B406:B407"/>
+    <mergeCell ref="B408:B409"/>
+    <mergeCell ref="B386:B387"/>
+    <mergeCell ref="B388:B389"/>
+    <mergeCell ref="B390:B391"/>
+    <mergeCell ref="B392:B393"/>
+    <mergeCell ref="B394:B395"/>
+    <mergeCell ref="B396:B397"/>
+    <mergeCell ref="B374:B375"/>
+    <mergeCell ref="B376:B377"/>
+    <mergeCell ref="B378:B379"/>
+    <mergeCell ref="B380:B381"/>
+    <mergeCell ref="B382:B383"/>
+    <mergeCell ref="B384:B385"/>
+    <mergeCell ref="B362:B363"/>
+    <mergeCell ref="B364:B365"/>
+    <mergeCell ref="B366:B367"/>
+    <mergeCell ref="B368:B369"/>
+    <mergeCell ref="B370:B371"/>
+    <mergeCell ref="B372:B373"/>
+    <mergeCell ref="B350:B351"/>
+    <mergeCell ref="B352:B353"/>
+    <mergeCell ref="B354:B355"/>
+    <mergeCell ref="B356:B357"/>
+    <mergeCell ref="B358:B359"/>
+    <mergeCell ref="B360:B361"/>
+    <mergeCell ref="B338:B339"/>
+    <mergeCell ref="B340:B341"/>
+    <mergeCell ref="B342:B343"/>
+    <mergeCell ref="B344:B345"/>
+    <mergeCell ref="B346:B347"/>
+    <mergeCell ref="B348:B349"/>
+    <mergeCell ref="B326:B327"/>
+    <mergeCell ref="B328:B329"/>
+    <mergeCell ref="B330:B331"/>
+    <mergeCell ref="B332:B333"/>
+    <mergeCell ref="B334:B335"/>
+    <mergeCell ref="B336:B337"/>
+    <mergeCell ref="B314:B315"/>
+    <mergeCell ref="B316:B317"/>
+    <mergeCell ref="B318:B319"/>
+    <mergeCell ref="B320:B321"/>
+    <mergeCell ref="B322:B323"/>
+    <mergeCell ref="B324:B325"/>
+    <mergeCell ref="B302:B303"/>
+    <mergeCell ref="B304:B305"/>
+    <mergeCell ref="B306:B307"/>
+    <mergeCell ref="B308:B309"/>
+    <mergeCell ref="B310:B311"/>
+    <mergeCell ref="B312:B313"/>
+    <mergeCell ref="B290:B291"/>
+    <mergeCell ref="B292:B293"/>
+    <mergeCell ref="B294:B295"/>
+    <mergeCell ref="B296:B297"/>
+    <mergeCell ref="B298:B299"/>
+    <mergeCell ref="B300:B301"/>
+    <mergeCell ref="B278:B279"/>
+    <mergeCell ref="B280:B281"/>
+    <mergeCell ref="B282:B283"/>
+    <mergeCell ref="B284:B285"/>
+    <mergeCell ref="B286:B287"/>
+    <mergeCell ref="B288:B289"/>
+    <mergeCell ref="B266:B267"/>
+    <mergeCell ref="B268:B269"/>
+    <mergeCell ref="B270:B271"/>
+    <mergeCell ref="B272:B273"/>
+    <mergeCell ref="B274:B275"/>
+    <mergeCell ref="B276:B277"/>
+    <mergeCell ref="B254:B255"/>
+    <mergeCell ref="B256:B257"/>
+    <mergeCell ref="B258:B259"/>
+    <mergeCell ref="B260:B261"/>
+    <mergeCell ref="B262:B263"/>
+    <mergeCell ref="B264:B265"/>
+    <mergeCell ref="B242:B243"/>
+    <mergeCell ref="B244:B245"/>
+    <mergeCell ref="B246:B247"/>
+    <mergeCell ref="B248:B249"/>
+    <mergeCell ref="B250:B251"/>
+    <mergeCell ref="B252:B253"/>
+    <mergeCell ref="B230:B231"/>
+    <mergeCell ref="B232:B233"/>
+    <mergeCell ref="B234:B235"/>
+    <mergeCell ref="B236:B237"/>
+    <mergeCell ref="B238:B239"/>
+    <mergeCell ref="B240:B241"/>
+    <mergeCell ref="B218:B219"/>
+    <mergeCell ref="B220:B221"/>
+    <mergeCell ref="B222:B223"/>
+    <mergeCell ref="B224:B225"/>
+    <mergeCell ref="B226:B227"/>
+    <mergeCell ref="B228:B229"/>
+    <mergeCell ref="B206:B207"/>
+    <mergeCell ref="B208:B209"/>
+    <mergeCell ref="B210:B211"/>
+    <mergeCell ref="B212:B213"/>
+    <mergeCell ref="B214:B215"/>
+    <mergeCell ref="B216:B217"/>
+    <mergeCell ref="B194:B195"/>
+    <mergeCell ref="B196:B197"/>
+    <mergeCell ref="B198:B199"/>
+    <mergeCell ref="B200:B201"/>
+    <mergeCell ref="B202:B203"/>
+    <mergeCell ref="B204:B205"/>
+    <mergeCell ref="B182:B183"/>
+    <mergeCell ref="B184:B185"/>
+    <mergeCell ref="B186:B187"/>
+    <mergeCell ref="B188:B189"/>
+    <mergeCell ref="B190:B191"/>
+    <mergeCell ref="B192:B193"/>
+    <mergeCell ref="B170:B171"/>
+    <mergeCell ref="B172:B173"/>
+    <mergeCell ref="B174:B175"/>
+    <mergeCell ref="B176:B177"/>
+    <mergeCell ref="B178:B179"/>
+    <mergeCell ref="B180:B181"/>
+    <mergeCell ref="B158:B159"/>
+    <mergeCell ref="B160:B161"/>
+    <mergeCell ref="B162:B163"/>
+    <mergeCell ref="B164:B165"/>
+    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="B168:B169"/>
+    <mergeCell ref="B146:B147"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="B152:B153"/>
+    <mergeCell ref="B154:B155"/>
+    <mergeCell ref="B156:B157"/>
+    <mergeCell ref="B134:B135"/>
+    <mergeCell ref="B136:B137"/>
+    <mergeCell ref="B138:B139"/>
+    <mergeCell ref="B140:B141"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="B144:B145"/>
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="B124:B125"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="B128:B129"/>
+    <mergeCell ref="B130:B131"/>
+    <mergeCell ref="B132:B133"/>
+    <mergeCell ref="B110:B111"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="B114:B115"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="B118:B119"/>
+    <mergeCell ref="B120:B121"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="B100:B101"/>
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="B104:B105"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="B108:B109"/>
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="B88:B89"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="B96:B97"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="B76:B77"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="B80:B81"/>
+    <mergeCell ref="B82:B83"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B36:B37"/>
     <mergeCell ref="B14:B15"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="B18:B19"/>
@@ -36994,544 +37532,6 @@
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="B86:B87"/>
-    <mergeCell ref="B88:B89"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="B96:B97"/>
-    <mergeCell ref="B74:B75"/>
-    <mergeCell ref="B76:B77"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="B80:B81"/>
-    <mergeCell ref="B82:B83"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="B110:B111"/>
-    <mergeCell ref="B112:B113"/>
-    <mergeCell ref="B114:B115"/>
-    <mergeCell ref="B116:B117"/>
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="B120:B121"/>
-    <mergeCell ref="B98:B99"/>
-    <mergeCell ref="B100:B101"/>
-    <mergeCell ref="B102:B103"/>
-    <mergeCell ref="B104:B105"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="B108:B109"/>
-    <mergeCell ref="B134:B135"/>
-    <mergeCell ref="B136:B137"/>
-    <mergeCell ref="B138:B139"/>
-    <mergeCell ref="B140:B141"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="B144:B145"/>
-    <mergeCell ref="B122:B123"/>
-    <mergeCell ref="B124:B125"/>
-    <mergeCell ref="B126:B127"/>
-    <mergeCell ref="B128:B129"/>
-    <mergeCell ref="B130:B131"/>
-    <mergeCell ref="B132:B133"/>
-    <mergeCell ref="B158:B159"/>
-    <mergeCell ref="B160:B161"/>
-    <mergeCell ref="B162:B163"/>
-    <mergeCell ref="B164:B165"/>
-    <mergeCell ref="B166:B167"/>
-    <mergeCell ref="B168:B169"/>
-    <mergeCell ref="B146:B147"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="B152:B153"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="B156:B157"/>
-    <mergeCell ref="B182:B183"/>
-    <mergeCell ref="B184:B185"/>
-    <mergeCell ref="B186:B187"/>
-    <mergeCell ref="B188:B189"/>
-    <mergeCell ref="B190:B191"/>
-    <mergeCell ref="B192:B193"/>
-    <mergeCell ref="B170:B171"/>
-    <mergeCell ref="B172:B173"/>
-    <mergeCell ref="B174:B175"/>
-    <mergeCell ref="B176:B177"/>
-    <mergeCell ref="B178:B179"/>
-    <mergeCell ref="B180:B181"/>
-    <mergeCell ref="B206:B207"/>
-    <mergeCell ref="B208:B209"/>
-    <mergeCell ref="B210:B211"/>
-    <mergeCell ref="B212:B213"/>
-    <mergeCell ref="B214:B215"/>
-    <mergeCell ref="B216:B217"/>
-    <mergeCell ref="B194:B195"/>
-    <mergeCell ref="B196:B197"/>
-    <mergeCell ref="B198:B199"/>
-    <mergeCell ref="B200:B201"/>
-    <mergeCell ref="B202:B203"/>
-    <mergeCell ref="B204:B205"/>
-    <mergeCell ref="B230:B231"/>
-    <mergeCell ref="B232:B233"/>
-    <mergeCell ref="B234:B235"/>
-    <mergeCell ref="B236:B237"/>
-    <mergeCell ref="B238:B239"/>
-    <mergeCell ref="B240:B241"/>
-    <mergeCell ref="B218:B219"/>
-    <mergeCell ref="B220:B221"/>
-    <mergeCell ref="B222:B223"/>
-    <mergeCell ref="B224:B225"/>
-    <mergeCell ref="B226:B227"/>
-    <mergeCell ref="B228:B229"/>
-    <mergeCell ref="B254:B255"/>
-    <mergeCell ref="B256:B257"/>
-    <mergeCell ref="B258:B259"/>
-    <mergeCell ref="B260:B261"/>
-    <mergeCell ref="B262:B263"/>
-    <mergeCell ref="B264:B265"/>
-    <mergeCell ref="B242:B243"/>
-    <mergeCell ref="B244:B245"/>
-    <mergeCell ref="B246:B247"/>
-    <mergeCell ref="B248:B249"/>
-    <mergeCell ref="B250:B251"/>
-    <mergeCell ref="B252:B253"/>
-    <mergeCell ref="B278:B279"/>
-    <mergeCell ref="B280:B281"/>
-    <mergeCell ref="B282:B283"/>
-    <mergeCell ref="B284:B285"/>
-    <mergeCell ref="B286:B287"/>
-    <mergeCell ref="B288:B289"/>
-    <mergeCell ref="B266:B267"/>
-    <mergeCell ref="B268:B269"/>
-    <mergeCell ref="B270:B271"/>
-    <mergeCell ref="B272:B273"/>
-    <mergeCell ref="B274:B275"/>
-    <mergeCell ref="B276:B277"/>
-    <mergeCell ref="B302:B303"/>
-    <mergeCell ref="B304:B305"/>
-    <mergeCell ref="B306:B307"/>
-    <mergeCell ref="B308:B309"/>
-    <mergeCell ref="B310:B311"/>
-    <mergeCell ref="B312:B313"/>
-    <mergeCell ref="B290:B291"/>
-    <mergeCell ref="B292:B293"/>
-    <mergeCell ref="B294:B295"/>
-    <mergeCell ref="B296:B297"/>
-    <mergeCell ref="B298:B299"/>
-    <mergeCell ref="B300:B301"/>
-    <mergeCell ref="B326:B327"/>
-    <mergeCell ref="B328:B329"/>
-    <mergeCell ref="B330:B331"/>
-    <mergeCell ref="B332:B333"/>
-    <mergeCell ref="B334:B335"/>
-    <mergeCell ref="B336:B337"/>
-    <mergeCell ref="B314:B315"/>
-    <mergeCell ref="B316:B317"/>
-    <mergeCell ref="B318:B319"/>
-    <mergeCell ref="B320:B321"/>
-    <mergeCell ref="B322:B323"/>
-    <mergeCell ref="B324:B325"/>
-    <mergeCell ref="B350:B351"/>
-    <mergeCell ref="B352:B353"/>
-    <mergeCell ref="B354:B355"/>
-    <mergeCell ref="B356:B357"/>
-    <mergeCell ref="B358:B359"/>
-    <mergeCell ref="B360:B361"/>
-    <mergeCell ref="B338:B339"/>
-    <mergeCell ref="B340:B341"/>
-    <mergeCell ref="B342:B343"/>
-    <mergeCell ref="B344:B345"/>
-    <mergeCell ref="B346:B347"/>
-    <mergeCell ref="B348:B349"/>
-    <mergeCell ref="B374:B375"/>
-    <mergeCell ref="B376:B377"/>
-    <mergeCell ref="B378:B379"/>
-    <mergeCell ref="B380:B381"/>
-    <mergeCell ref="B382:B383"/>
-    <mergeCell ref="B384:B385"/>
-    <mergeCell ref="B362:B363"/>
-    <mergeCell ref="B364:B365"/>
-    <mergeCell ref="B366:B367"/>
-    <mergeCell ref="B368:B369"/>
-    <mergeCell ref="B370:B371"/>
-    <mergeCell ref="B372:B373"/>
-    <mergeCell ref="B398:B399"/>
-    <mergeCell ref="B400:B401"/>
-    <mergeCell ref="B402:B403"/>
-    <mergeCell ref="B404:B405"/>
-    <mergeCell ref="B406:B407"/>
-    <mergeCell ref="B408:B409"/>
-    <mergeCell ref="B386:B387"/>
-    <mergeCell ref="B388:B389"/>
-    <mergeCell ref="B390:B391"/>
-    <mergeCell ref="B392:B393"/>
-    <mergeCell ref="B394:B395"/>
-    <mergeCell ref="B396:B397"/>
-    <mergeCell ref="B422:B423"/>
-    <mergeCell ref="B424:B425"/>
-    <mergeCell ref="B426:B427"/>
-    <mergeCell ref="B428:B429"/>
-    <mergeCell ref="B430:B431"/>
-    <mergeCell ref="B432:B433"/>
-    <mergeCell ref="B410:B411"/>
-    <mergeCell ref="B412:B413"/>
-    <mergeCell ref="B414:B415"/>
-    <mergeCell ref="B416:B417"/>
-    <mergeCell ref="B418:B419"/>
-    <mergeCell ref="B420:B421"/>
-    <mergeCell ref="B446:B447"/>
-    <mergeCell ref="B448:B449"/>
-    <mergeCell ref="B450:B451"/>
-    <mergeCell ref="B452:B453"/>
-    <mergeCell ref="B454:B455"/>
-    <mergeCell ref="B456:B457"/>
-    <mergeCell ref="B434:B435"/>
-    <mergeCell ref="B436:B437"/>
-    <mergeCell ref="B438:B439"/>
-    <mergeCell ref="B440:B441"/>
-    <mergeCell ref="B442:B443"/>
-    <mergeCell ref="B444:B445"/>
-    <mergeCell ref="B470:B471"/>
-    <mergeCell ref="B472:B473"/>
-    <mergeCell ref="B474:B475"/>
-    <mergeCell ref="B476:B477"/>
-    <mergeCell ref="B478:B479"/>
-    <mergeCell ref="B480:B481"/>
-    <mergeCell ref="B458:B459"/>
-    <mergeCell ref="B460:B461"/>
-    <mergeCell ref="B462:B463"/>
-    <mergeCell ref="B464:B465"/>
-    <mergeCell ref="B466:B467"/>
-    <mergeCell ref="B468:B469"/>
-    <mergeCell ref="B494:B495"/>
-    <mergeCell ref="B496:B497"/>
-    <mergeCell ref="B498:B499"/>
-    <mergeCell ref="B500:B501"/>
-    <mergeCell ref="B502:B503"/>
-    <mergeCell ref="B504:B505"/>
-    <mergeCell ref="B482:B483"/>
-    <mergeCell ref="B484:B485"/>
-    <mergeCell ref="B486:B487"/>
-    <mergeCell ref="B488:B489"/>
-    <mergeCell ref="B490:B491"/>
-    <mergeCell ref="B492:B493"/>
-    <mergeCell ref="B518:B519"/>
-    <mergeCell ref="B520:B521"/>
-    <mergeCell ref="B522:B523"/>
-    <mergeCell ref="B524:B525"/>
-    <mergeCell ref="B526:B527"/>
-    <mergeCell ref="B528:B529"/>
-    <mergeCell ref="B506:B507"/>
-    <mergeCell ref="B508:B509"/>
-    <mergeCell ref="B510:B511"/>
-    <mergeCell ref="B512:B513"/>
-    <mergeCell ref="B514:B515"/>
-    <mergeCell ref="B516:B517"/>
-    <mergeCell ref="B542:B543"/>
-    <mergeCell ref="B544:B545"/>
-    <mergeCell ref="B546:B547"/>
-    <mergeCell ref="B548:B549"/>
-    <mergeCell ref="B550:B551"/>
-    <mergeCell ref="B552:B553"/>
-    <mergeCell ref="B530:B531"/>
-    <mergeCell ref="B532:B533"/>
-    <mergeCell ref="B534:B535"/>
-    <mergeCell ref="B536:B537"/>
-    <mergeCell ref="B538:B539"/>
-    <mergeCell ref="B540:B541"/>
-    <mergeCell ref="B566:B567"/>
-    <mergeCell ref="B568:B569"/>
-    <mergeCell ref="B570:B571"/>
-    <mergeCell ref="B572:B573"/>
-    <mergeCell ref="B574:B575"/>
-    <mergeCell ref="B576:B577"/>
-    <mergeCell ref="B554:B555"/>
-    <mergeCell ref="B556:B557"/>
-    <mergeCell ref="B558:B559"/>
-    <mergeCell ref="B560:B561"/>
-    <mergeCell ref="B562:B563"/>
-    <mergeCell ref="B564:B565"/>
-    <mergeCell ref="B590:B591"/>
-    <mergeCell ref="B592:B593"/>
-    <mergeCell ref="B594:B595"/>
-    <mergeCell ref="B596:B597"/>
-    <mergeCell ref="B598:B599"/>
-    <mergeCell ref="B600:B601"/>
-    <mergeCell ref="B578:B579"/>
-    <mergeCell ref="B580:B581"/>
-    <mergeCell ref="B582:B583"/>
-    <mergeCell ref="B584:B585"/>
-    <mergeCell ref="B586:B587"/>
-    <mergeCell ref="B588:B589"/>
-    <mergeCell ref="B614:B615"/>
-    <mergeCell ref="B616:B617"/>
-    <mergeCell ref="B618:B619"/>
-    <mergeCell ref="B620:B621"/>
-    <mergeCell ref="B622:B623"/>
-    <mergeCell ref="B624:B625"/>
-    <mergeCell ref="B602:B603"/>
-    <mergeCell ref="B604:B605"/>
-    <mergeCell ref="B606:B607"/>
-    <mergeCell ref="B608:B609"/>
-    <mergeCell ref="B610:B611"/>
-    <mergeCell ref="B612:B613"/>
-    <mergeCell ref="B638:B639"/>
-    <mergeCell ref="B640:B641"/>
-    <mergeCell ref="B642:B643"/>
-    <mergeCell ref="B644:B645"/>
-    <mergeCell ref="B646:B647"/>
-    <mergeCell ref="B648:B649"/>
-    <mergeCell ref="B626:B627"/>
-    <mergeCell ref="B628:B629"/>
-    <mergeCell ref="B630:B631"/>
-    <mergeCell ref="B632:B633"/>
-    <mergeCell ref="B634:B635"/>
-    <mergeCell ref="B636:B637"/>
-    <mergeCell ref="B662:B663"/>
-    <mergeCell ref="B664:B665"/>
-    <mergeCell ref="B666:B667"/>
-    <mergeCell ref="B668:B669"/>
-    <mergeCell ref="B670:B671"/>
-    <mergeCell ref="B672:B673"/>
-    <mergeCell ref="B650:B651"/>
-    <mergeCell ref="B652:B653"/>
-    <mergeCell ref="B654:B655"/>
-    <mergeCell ref="B656:B657"/>
-    <mergeCell ref="B658:B659"/>
-    <mergeCell ref="B660:B661"/>
-    <mergeCell ref="B686:B687"/>
-    <mergeCell ref="B688:B689"/>
-    <mergeCell ref="B690:B691"/>
-    <mergeCell ref="B692:B693"/>
-    <mergeCell ref="B694:B695"/>
-    <mergeCell ref="B696:B697"/>
-    <mergeCell ref="B674:B675"/>
-    <mergeCell ref="B676:B677"/>
-    <mergeCell ref="B678:B679"/>
-    <mergeCell ref="B680:B681"/>
-    <mergeCell ref="B682:B683"/>
-    <mergeCell ref="B684:B685"/>
-    <mergeCell ref="B710:B711"/>
-    <mergeCell ref="B712:B713"/>
-    <mergeCell ref="B714:B715"/>
-    <mergeCell ref="B716:B717"/>
-    <mergeCell ref="B718:B719"/>
-    <mergeCell ref="B720:B721"/>
-    <mergeCell ref="B698:B699"/>
-    <mergeCell ref="B700:B701"/>
-    <mergeCell ref="B702:B703"/>
-    <mergeCell ref="B704:B705"/>
-    <mergeCell ref="B706:B707"/>
-    <mergeCell ref="B708:B709"/>
-    <mergeCell ref="B734:B735"/>
-    <mergeCell ref="B736:B737"/>
-    <mergeCell ref="B738:B739"/>
-    <mergeCell ref="B740:B741"/>
-    <mergeCell ref="B742:B743"/>
-    <mergeCell ref="B744:B745"/>
-    <mergeCell ref="B722:B723"/>
-    <mergeCell ref="B724:B725"/>
-    <mergeCell ref="B726:B727"/>
-    <mergeCell ref="B728:B729"/>
-    <mergeCell ref="B730:B731"/>
-    <mergeCell ref="B732:B733"/>
-    <mergeCell ref="B758:B759"/>
-    <mergeCell ref="B760:B761"/>
-    <mergeCell ref="B762:B763"/>
-    <mergeCell ref="B764:B765"/>
-    <mergeCell ref="B766:B767"/>
-    <mergeCell ref="B768:B769"/>
-    <mergeCell ref="B746:B747"/>
-    <mergeCell ref="B748:B749"/>
-    <mergeCell ref="B750:B751"/>
-    <mergeCell ref="B752:B753"/>
-    <mergeCell ref="B754:B755"/>
-    <mergeCell ref="B756:B757"/>
-    <mergeCell ref="B782:B783"/>
-    <mergeCell ref="B784:B785"/>
-    <mergeCell ref="B786:B787"/>
-    <mergeCell ref="B788:B789"/>
-    <mergeCell ref="B790:B791"/>
-    <mergeCell ref="B792:B793"/>
-    <mergeCell ref="B770:B771"/>
-    <mergeCell ref="B772:B773"/>
-    <mergeCell ref="B774:B775"/>
-    <mergeCell ref="B776:B777"/>
-    <mergeCell ref="B778:B779"/>
-    <mergeCell ref="B780:B781"/>
-    <mergeCell ref="B806:B807"/>
-    <mergeCell ref="B808:B809"/>
-    <mergeCell ref="B810:B811"/>
-    <mergeCell ref="B812:B813"/>
-    <mergeCell ref="B814:B815"/>
-    <mergeCell ref="B816:B817"/>
-    <mergeCell ref="B794:B795"/>
-    <mergeCell ref="B796:B797"/>
-    <mergeCell ref="B798:B799"/>
-    <mergeCell ref="B800:B801"/>
-    <mergeCell ref="B802:B803"/>
-    <mergeCell ref="B804:B805"/>
-    <mergeCell ref="B830:B831"/>
-    <mergeCell ref="B832:B833"/>
-    <mergeCell ref="B834:B835"/>
-    <mergeCell ref="B836:B837"/>
-    <mergeCell ref="B838:B839"/>
-    <mergeCell ref="B840:B841"/>
-    <mergeCell ref="B818:B819"/>
-    <mergeCell ref="B820:B821"/>
-    <mergeCell ref="B822:B823"/>
-    <mergeCell ref="B824:B825"/>
-    <mergeCell ref="B826:B827"/>
-    <mergeCell ref="B828:B829"/>
-    <mergeCell ref="B854:B855"/>
-    <mergeCell ref="B856:B857"/>
-    <mergeCell ref="B858:B859"/>
-    <mergeCell ref="B860:B861"/>
-    <mergeCell ref="B862:B863"/>
-    <mergeCell ref="B864:B865"/>
-    <mergeCell ref="B842:B843"/>
-    <mergeCell ref="B844:B845"/>
-    <mergeCell ref="B846:B847"/>
-    <mergeCell ref="B848:B849"/>
-    <mergeCell ref="B850:B851"/>
-    <mergeCell ref="B852:B853"/>
-    <mergeCell ref="B878:B879"/>
-    <mergeCell ref="B880:B881"/>
-    <mergeCell ref="B882:B883"/>
-    <mergeCell ref="B884:B885"/>
-    <mergeCell ref="B886:B887"/>
-    <mergeCell ref="B888:B889"/>
-    <mergeCell ref="B866:B867"/>
-    <mergeCell ref="B868:B869"/>
-    <mergeCell ref="B870:B871"/>
-    <mergeCell ref="B872:B873"/>
-    <mergeCell ref="B874:B875"/>
-    <mergeCell ref="B876:B877"/>
-    <mergeCell ref="B902:B903"/>
-    <mergeCell ref="B904:B905"/>
-    <mergeCell ref="B906:B907"/>
-    <mergeCell ref="B908:B909"/>
-    <mergeCell ref="B910:B911"/>
-    <mergeCell ref="B912:B913"/>
-    <mergeCell ref="B890:B891"/>
-    <mergeCell ref="B892:B893"/>
-    <mergeCell ref="B894:B895"/>
-    <mergeCell ref="B896:B897"/>
-    <mergeCell ref="B898:B899"/>
-    <mergeCell ref="B900:B901"/>
-    <mergeCell ref="B926:B927"/>
-    <mergeCell ref="B928:B929"/>
-    <mergeCell ref="B930:B931"/>
-    <mergeCell ref="B932:B933"/>
-    <mergeCell ref="B934:B935"/>
-    <mergeCell ref="B936:B937"/>
-    <mergeCell ref="B914:B915"/>
-    <mergeCell ref="B916:B917"/>
-    <mergeCell ref="B918:B919"/>
-    <mergeCell ref="B920:B921"/>
-    <mergeCell ref="B922:B923"/>
-    <mergeCell ref="B924:B925"/>
-    <mergeCell ref="B950:B951"/>
-    <mergeCell ref="B952:B953"/>
-    <mergeCell ref="B954:B955"/>
-    <mergeCell ref="B956:B957"/>
-    <mergeCell ref="B958:B959"/>
-    <mergeCell ref="B960:B961"/>
-    <mergeCell ref="B938:B939"/>
-    <mergeCell ref="B940:B941"/>
-    <mergeCell ref="B942:B943"/>
-    <mergeCell ref="B944:B945"/>
-    <mergeCell ref="B946:B947"/>
-    <mergeCell ref="B948:B949"/>
-    <mergeCell ref="B974:B975"/>
-    <mergeCell ref="B976:B977"/>
-    <mergeCell ref="B978:B979"/>
-    <mergeCell ref="B980:B981"/>
-    <mergeCell ref="B982:B983"/>
-    <mergeCell ref="B984:B985"/>
-    <mergeCell ref="B962:B963"/>
-    <mergeCell ref="B964:B965"/>
-    <mergeCell ref="B966:B967"/>
-    <mergeCell ref="B968:B969"/>
-    <mergeCell ref="B970:B971"/>
-    <mergeCell ref="B972:B973"/>
-    <mergeCell ref="B998:B999"/>
-    <mergeCell ref="B1000:B1001"/>
-    <mergeCell ref="B1002:B1003"/>
-    <mergeCell ref="B1004:B1005"/>
-    <mergeCell ref="B1006:B1007"/>
-    <mergeCell ref="B1008:B1009"/>
-    <mergeCell ref="B986:B987"/>
-    <mergeCell ref="B988:B989"/>
-    <mergeCell ref="B990:B991"/>
-    <mergeCell ref="B992:B993"/>
-    <mergeCell ref="B994:B995"/>
-    <mergeCell ref="B996:B997"/>
-    <mergeCell ref="B1022:B1023"/>
-    <mergeCell ref="B1024:B1025"/>
-    <mergeCell ref="B1026:B1027"/>
-    <mergeCell ref="B1028:B1029"/>
-    <mergeCell ref="B1030:B1031"/>
-    <mergeCell ref="B1032:B1033"/>
-    <mergeCell ref="B1010:B1011"/>
-    <mergeCell ref="B1012:B1013"/>
-    <mergeCell ref="B1014:B1015"/>
-    <mergeCell ref="B1016:B1017"/>
-    <mergeCell ref="B1018:B1019"/>
-    <mergeCell ref="B1020:B1021"/>
-    <mergeCell ref="B1046:B1047"/>
-    <mergeCell ref="B1048:B1049"/>
-    <mergeCell ref="B1050:B1051"/>
-    <mergeCell ref="B1052:B1053"/>
-    <mergeCell ref="B1054:B1055"/>
-    <mergeCell ref="B1056:B1057"/>
-    <mergeCell ref="B1034:B1035"/>
-    <mergeCell ref="B1036:B1037"/>
-    <mergeCell ref="B1038:B1039"/>
-    <mergeCell ref="B1040:B1041"/>
-    <mergeCell ref="B1042:B1043"/>
-    <mergeCell ref="B1044:B1045"/>
-    <mergeCell ref="B1070:B1071"/>
-    <mergeCell ref="B1072:B1073"/>
-    <mergeCell ref="B1074:B1075"/>
-    <mergeCell ref="B1076:B1077"/>
-    <mergeCell ref="B1078:B1079"/>
-    <mergeCell ref="B1080:B1081"/>
-    <mergeCell ref="B1058:B1059"/>
-    <mergeCell ref="B1060:B1061"/>
-    <mergeCell ref="B1062:B1063"/>
-    <mergeCell ref="B1064:B1065"/>
-    <mergeCell ref="B1066:B1067"/>
-    <mergeCell ref="B1068:B1069"/>
-    <mergeCell ref="B1094:B1095"/>
-    <mergeCell ref="B1096:B1097"/>
-    <mergeCell ref="B1098:B1099"/>
-    <mergeCell ref="B1100:B1101"/>
-    <mergeCell ref="B1082:B1083"/>
-    <mergeCell ref="B1084:B1085"/>
-    <mergeCell ref="B1086:B1087"/>
-    <mergeCell ref="B1088:B1089"/>
-    <mergeCell ref="B1090:B1091"/>
-    <mergeCell ref="B1092:B1093"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix incorrect function params caused by use of var instead of let
</commit_message>
<xml_diff>
--- a/demo/demo.xlsx
+++ b/demo/demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\~\Webcellar\demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0882E67A-4792-4388-A38E-02984E5EE50E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B76E7C-7848-401B-9F9A-349AE5922213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ECFAADD7-15DE-4BAC-B94D-A5FD0FC4859A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ECFAADD7-15DE-4BAC-B94D-A5FD0FC4859A}"/>
   </bookViews>
   <sheets>
     <sheet name="Demo" sheetId="1" r:id="rId1"/>
@@ -113,7 +113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>A.STRING()</t>
   </si>
@@ -212,6 +212,12 @@
   </si>
   <si>
     <t>A.FOO()</t>
+  </si>
+  <si>
+    <t>ZZZ()</t>
+  </si>
+  <si>
+    <t>ZZZ.A()</t>
   </si>
 </sst>
 </file>
@@ -352,21 +358,23 @@
     <v>six</v>
   </rv>
   <rv s="4">
-    <v>14</v>
-  </rv>
-  <rv s="5">
     <v>Car</v>
     <v>BMW</v>
     <v>120</v>
   </rv>
-  <rv s="5">
+  <rv s="4">
     <v>Car</v>
     <v>Ferrari</v>
     <v>9000</v>
   </rv>
-  <rv s="6">
+  <rv s="5">
     <v>Foo</v>
     <v>https://localhost:29640/C:/~/Webcellar/demo/foo/foo.xlsx.js</v>
+  </rv>
+  <rv s="6">
+    <v/>
+    <v>Hello</v>
+    <v>World!</v>
   </rv>
 </rvData>
 </file>
@@ -393,9 +401,6 @@
     <k n="c" t="r"/>
     <k n="e" t="s"/>
   </s>
-  <s t="_error">
-    <k n="errorType" t="i"/>
-  </s>
   <s t="_entity">
     <k n="_DisplayString" t="s"/>
     <k n="brand" t="s"/>
@@ -404,6 +409,11 @@
   <s t="_entity">
     <k n="_DisplayString" t="s"/>
     <k n="url" t="s"/>
+  </s>
+  <s t="_entity">
+    <k n="_DisplayString" t="s"/>
+    <k n="a" t="s"/>
+    <k n="b" t="s"/>
   </s>
 </rvStructures>
 </file>
@@ -746,6 +756,9 @@
     </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_A_ZZZ</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_A_ZZZ_B</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_A_ZZZ_A</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_A_VOLATILESTATEFULRANDOMWALK</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_A_TIMESTAMP</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_A_TEST</we:customFunctionIds>
@@ -784,7 +797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60D5786C-8346-49E1-951B-BC797AA7FCE3}">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="2" bestFit="1" customWidth="1"/>
@@ -1032,7 +1045,7 @@
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" cm="1">
         <f t="array" aca="1" ref="A45" ca="1">_xldudf_A_VOLATILESTATEFULRANDOMWALK()</f>
-        <v>0.54148105686912151</v>
+        <v>1385.3511466605692</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1055,7 +1068,7 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="e" cm="1" vm="3">
+      <c r="A51" s="2" t="e" cm="1" vm="2">
         <f t="array" ref="A51">_xldudf_A_CAR("BMW", 120)</f>
         <v>#VALUE!</v>
       </c>
@@ -1069,7 +1082,7 @@
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="e" cm="1" vm="4">
+      <c r="A54" s="2" t="e" cm="1" vm="3">
         <f t="array" ref="A54">_xldudf_A_CARINSTANCE()</f>
         <v>#VALUE!</v>
       </c>
@@ -1091,9 +1104,9 @@
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="e" cm="1">
-        <f t="array" aca="1" ref="A60" ca="1">_xldudf_A_TIMESTAMP(TRUE)</f>
-        <v>#NAME?</v>
+      <c r="A60" s="2" t="str" cm="1">
+        <f t="array" ref="A60">_xldudf_A_TIMESTAMP(TRUE)</f>
+        <v>Mon, 13 Apr 2026 02:20:39 GMT</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1113,9 +1126,31 @@
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" s="2" t="e" cm="1" vm="5">
+      <c r="A66" s="2" t="e" cm="1" vm="4">
         <f t="array" ref="A66">_xldudf_A_FOO()</f>
         <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="e" cm="1" vm="5">
+        <f t="array" ref="A69">_xldudf_ZZZ()</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="str" cm="1">
+        <f t="array" ref="A72">_xldudf_ZZZ_A()</f>
+        <v>Hello</v>
       </c>
     </row>
   </sheetData>

</xml_diff>